<commit_message>
Refresh Banking content for SOP 50 10 8.1 on October 1, 2026.
Update live SBA copy, dates, and quick-check notes, and replace the published Banking downloads with the rebuilt templates.

Co-authored-by: bkchiesa <bkchiesa@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/public/downloads/banking/cash-flow-projection-12mo.xlsx
+++ b/public/downloads/banking/cash-flow-projection-12mo.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Blank template" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Example" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Instructions" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Blank template" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Example" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
Banking Oct 2026 annual refresh (SOP 50 10 8.1)
Update live SBA copy, dates, and quick-check notes, and replace the published Banking downloads with the rebuilt templates.

Co-authored-by: Cursor Agent <cursoragent@cursor.com>
Co-authored-by: bkchiesa <bkchiesa@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/public/downloads/banking/cash-flow-projection-12mo.xlsx
+++ b/public/downloads/banking/cash-flow-projection-12mo.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Blank template" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Example" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Instructions" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Blank template" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Example" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>